<commit_message>
update to parse windows printer 2
</commit_message>
<xml_diff>
--- a/SessionBackup/LastSessionItems.xlsx
+++ b/SessionBackup/LastSessionItems.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan\Desktop\barcodeutils\SessionBackup\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sann juan 2\Desktop\barcodeUtils-master\SessionBackup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1A81F74-C9D0-4E12-9FBE-4A17943DC5FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8C09DF5-D893-46B6-BDBE-0D2B7B776D65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="4290" windowWidth="28800" windowHeight="15435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6480" yWindow="4050" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Productos" sheetId="1" r:id="rId1"/>
@@ -16473,7 +16473,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja1"/>
   <dimension ref="A3:L4227"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">

</xml_diff>